<commit_message>
Aplica la evaluación de los agentes a la 3.2.4 y corrige el período de consultas
- 3.2.4: metodología con ejemplos de atomicidad (la regla de estructura canónica reescribe, no divide), MoSCoW explicado, 152 de prioridad alta desglosado (146 de la Etapa 1 y 6 de garantía legal), método de verificación acotado por tipo, Tabla 3.5 en lenguaje claro con las cifras del catálogo, versión del catálogo en la fuente.
- El período de consultas ya cerró (art. 43 y T-20): lo que se consultaba al mandante o se validaba en ese período se valida ahora con el cliente al inicio del proyecto, antes de fijar la línea base (3.2.3, 3.2.4, anexos y Excel v3.1).
- Comité Ejecutivo pasa a «del contrato» (art. 71).
- Se mantiene el T-12 como lugar de la correspondencia con los requisitos transversales; no se agrega columna RT.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_Requerimientos/RequerimientosAtomizados_Depuracion_Alcance_v3.1.xlsx
+++ b/01_Requerimientos/RequerimientosAtomizados_Depuracion_Alcance_v3.1.xlsx
@@ -346,7 +346,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RF-227 a RF-231, propuestos para el servicio de clientes Retail, que no tenía requerimientos. Por validar en el período de consultas.</t>
+          <t xml:space="preserve">RF-227 a RF-231, propuestos para el servicio de clientes Retail, que no tenía requerimientos. Por validar con el cliente al inicio del proyecto.</t>
         </is>
       </c>
     </row>
@@ -20126,7 +20126,7 @@
       </c>
       <c r="M256" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se eleva de 4 a 24 horas: RT-03.10 y el art. 16.4 no admiten menos de 24 horas para el componente on-premise. El valor de 4 horas del Caso queda por debajo y rige el más exigente. Se consulta al mandante.</t>
+          <t xml:space="preserve">Se eleva de 4 a 24 horas: RT-03.10 y el art. 16.4 no admiten menos de 24 horas para el componente on-premise. El valor de 4 horas del Caso queda por debajo y rige el más exigente. Se valida con el cliente al inicio del proyecto, antes de fijar la línea base.</t>
         </is>
       </c>
       <c r="N256" s="6" t="inlineStr">
@@ -26563,7 +26563,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inventario de flujos autorizados; todo intento no declarado queda bloqueado y registrado. Auditoría (ventana por definir en el período de consultas) sobre 100 % de los cruces.</t>
+          <t xml:space="preserve">Inventario de flujos autorizados; todo intento no declarado queda bloqueado y registrado. Auditoría (ventana por definir con el cliente al inicio del proyecto) sobre 100 % de los cruces.</t>
         </is>
       </c>
     </row>
@@ -30069,7 +30069,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nueve filas con «??» sin confirmar (hallazgo H-19) y 16 supuestos por umbrales ausentes: se llevan al período de consultas.</t>
+          <t xml:space="preserve">Nueve filas con «??» sin confirmar (hallazgo H-19) y 16 supuestos por umbrales ausentes: se validan con el cliente al inicio del proyecto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cierra la 3.2.5 con el Anexo D, ajusta la 3.1 y reorganiza el contexto del sd-03
Reescribe la 3.2.5 con tres niveles de aceptación y la Tabla 3.6, tras dos
rondas de los agentes. Crea el Anexo D (28 criterios) y su hoja en el Excel
v3.1. Corrige en la 3.1 los nombres de la evidencia financiera y la base
tecnológica. Agrega la ficha de alcance, el índice y el script de control de
desfase, y archiva el material superado como no_usar_*.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_Requerimientos/RequerimientosAtomizados_Depuracion_Alcance_v3.1.xlsx
+++ b/01_Requerimientos/RequerimientosAtomizados_Depuracion_Alcance_v3.1.xlsx
@@ -11,6 +11,7 @@
     <sheet name="6_Divisiones_v3.0" sheetId="7" r:id="rId7"/>
     <sheet name="7_Hallazgos_v3.0" sheetId="8" r:id="rId8"/>
     <sheet name="8_Pendientes" sheetId="9" r:id="rId9"/>
+    <sheet name="9_Criterios_Aceptacion" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1_Catalogo_Vigente'!$A$1:$O$309</definedName>
@@ -404,6 +405,1191 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="52" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N.º</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado esperado</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Línea base</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meta</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se alcanza</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evidencia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Responsabilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El disponible que se publica incorpora el error conocido del registro y se calcula por categoría y por punto.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suma de existencias menos un descuento fijo definido en 2019.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cálculo dinámico por categoría y punto (Caso, cap. 7), con tolerancia respecto del conteo por fijar al inicio del proyecto (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de existencias</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16, con despliegue gradual por categorías</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba del cálculo del disponible con el colchón de confianza por categoría y punto (RF-127 a RF-129).</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los pedidos cancelados por falta de existencia bajan al umbral comprometido, también durante el evento anual.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1,9 % en el año, 2,7 % en el evento y 2.840 casos en 3 días.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bajo 0,3 % al año y cero cancelaciones por falta de existencia durante el evento (Caso, cap. 7). Reclasificado desde RNF-61. Mes 16, solo categorías con existencias en producción, medida sin meta de cero. Mes 21, con pedidos, meta completa.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de existencias y de pedidos</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16 con existencias y primer evento anual posterior al mes 21 con pedidos</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medición mensual de las cancelaciones y medición en cada evento anual. La parte de la solución son las cancelaciones por falta de existencia o por disponible mal calculado. La parte del cliente son las cancelaciones por preparación de pedidos en tienda y centro de distribución.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compartida entre el proponente y el cliente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ningún cliente es cobrado por una unidad que la compañía no puede entregar.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se cobró y se devolvió ocho días después.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cero casos (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de pedidos y de existencias</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auditoría de los pedidos con cobro capturado sobre un pedido no cumplible (RNF-65).</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La exactitud del inventario se mide de forma continua y por categoría, contando sin cerrar la tienda.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conteo cíclico con 12,4 % de diferencia y sin desglose.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diferencia de conteo bajo 2 % (Caso, cap. 7). Reclasificado desde RNF-63.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de existencias</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16 con despliegue gradual por tienda y categoría, y mes 21 en las 22 tiendas</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conteo cíclico por categoría sin cerrar la tienda (RF-131 y RF-135) y exactitud diaria por categoría (RT-05.29). La parte de la solución es el registro y el cálculo de la exactitud. La parte del cliente es la ejecución del conteo en sala según la frecuencia acordada.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compartida entre el proponente y el cliente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La merma está separada en sus causas: pérdida física, daño, error de recepción, devolución mal reintegrada y error de digitación.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merma de 1,9 % de la venta, $ 7.800 millones al año, tratada como un solo problema.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de los ajustes con causa (propuesta del proponente) y merma bajo 1 % (Caso, cap. 7).</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de existencias</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe mensual de merma por causa, cuya suma de componentes es igual al total (RN-12 y RF-138).</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Un cambio de precio llega a las cajas, al canal digital y a la sala dentro del plazo comprometido.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cajas y sitio en minutos y etiqueta hasta 24 horas después.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 minutos o menos en cajas y canal digital (RT-09.01). En sala, por definir con la política de precios en sala.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de oferta comercial</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medición de la latencia de propagación por destino (RNF-19).</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La compañía sabe, en todo momento, cuántos puntos de exhibición están desactualizados y cuáles.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No existe registro de qué etiqueta se cambió ni cuándo.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de los puntos con estado registrado (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de oferta comercial</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indicador diario de puntos de exhibición desactualizados (RF-029).</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se puede acreditar qué precio estaba publicado en cada canal en un instante determinado.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inexistente. No se puede responder ni a favor ni en contra.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recuperación en 1 minuto o menos sobre una ventana de tres años (propuesta del proponente, RNF-44 y RNF-58).</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de oferta comercial</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consulta del precio publicado por fecha, hora y canal (RNF-58).</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El precio cobrado es el precio exhibido, verificado por muestreo propio y no por fiscalización externa.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11 % de discrepancia en la fiscalización de febrero.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0,5 % o menos, verificado por muestreo propio (propuesta del proponente). La política de precios en sala está pendiente (supuestos SUP-08 y SUP-09).</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de oferta comercial y de ventas</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Muestreo propio de precios cobrados y exhibidos por tienda. La parte de la solución es el precio publicado en cajas y canal digital. La parte del cliente es la etiqueta de sala en la tienda.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compartida entre el proponente y el cliente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Un pedido tiene un estado único, consultable por el cliente, la tienda, el mesón, el centro de distribución y el vendedor externo.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada canal ve un estado distinto y el mesón no ve los pedidos en línea.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado único y consistente en todos los canales (RT-05.29).</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de pedidos</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auditoría cruzada del estado del pedido entre canales (RF-052 y RNF-04).</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La decisión del punto de despacho considera el costo total y el efecto sobre la sala de venta.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se decide por distancia.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de las asignaciones con costo total (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de pedidos</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registro del costo total en cada asignación de despacho (RF-076 y RF-077).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La tienda que entrega una unidad para un pedido de otro canal recibe el reconocimiento correspondiente.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inexistente. La unidad a veces no aparece.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de los despachos desde tienda atribuidos (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de comisiones</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registro de la atribución de cada despacho (RF-071, con la base de comisión de RF-054 y RF-055).</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La devolución de un producto de marketplace tiene un procedimiento definido y el vendedor externo se entera cuando ocurre.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No hay regla escrita. El vendedor se entera en la liquidación.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aviso al vendedor en 15 minutos o menos en cada devolución (propuesta del proponente, RNF-66).</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de marketplace y de posventa</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registro del aviso al vendedor por cada devolución (RNF-66).</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los 310 vendedores de marketplace se evalúan con reglas que ellos conocen y que tienen consecuencia.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No hay acuerdo de nivel de servicio medido.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de los vendedores con nivel de servicio medido (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de marketplace</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21 y renovación anual de los acuerdos</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe mensual del nivel de servicio de cada vendedor, con las reglas conocidas por ellos (propuesta del proponente, RF-105, RF-112 y RF-119).</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La garantía legal se resuelve en el mesón sin derivar al cliente al fabricante ni al vendedor externo.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El proceso completo consiste en derivar.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cero derivaciones (restricción 7 del Caso).</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de posventa</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Programa de cliente oculto en las 22 tiendas (RNF-69). La parte de la solución es la herramienta de garantía en el mesón. La parte del cliente es la atención del mesón sin derivar.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compartida entre el proponente y el cliente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La evaluación crediticia en el punto de venta se resuelve en el umbral comprometido.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entre 40 segundos y 3 minutos.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 segundos o menos (RT-09.01 y RNF-06).</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de originación de crédito</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medición de extremo a extremo en el punto de venta (RNF-06).</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Queda registro estructurado de qué información precontractual se entregó, en qué versión y antes de la aceptación.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Una firma en un formulario que se archiva.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registro trazable por operación (Caso, cap. 7).</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registro de la versión, el instante y el medio de entrega por operación (RF-200 a RF-204).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ninguna repactación puede registrarse sin evidencia recuperable del consentimiento informado.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.240 casos de 2025 sin evidencia recuperable.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cero repactaciones sin evidencia (Caso, cap. 7).</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de cartera de crédito y de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16 para los actos nuevos y mes 21 con la cartera migrada</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba de bloqueo de una repactación sin evidencia y auditoría de los actos del período.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La evidencia del consentimiento se conserva y se recupera por el plazo del crédito y el período posterior exigido.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grabaciones conservadas 90 días.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plazo del crédito más seis años, con recuperación a diez años en 5 minutos o menos (propuesta del proponente, RNF-42, RNF-43 y RNF-57).</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulacro de requerimiento de la autoridad fiscalizadora (RNF-57).</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El cumplimiento de la entrega de información no depende de la voluntad del vendedor: el proceso impide omitirla.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Depende de que el vendedor tenga tiempo.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El proceso impide aceptar un crédito sin la información (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de originación de crédito y de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba negativa: el intento de aceptar sin la información completa es rechazado (RF-199 y RF-206).</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La separación entre los datos del retail y los de la filial emisora está implementada, documentada y auditada.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial y no documentada.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementada y documentada (Caso, cap. 7), con cero hallazgos críticos o altos en la prueba de penetración (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de control de cruces</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe técnico de separación y prueba de penetración (RNF-11 y RNF-14).</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todo cruce de información entre ambos ámbitos queda registrado con su finalidad, su base y su autorización.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No existe registro de cruces.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de los cruces registrados (RF-165).</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de control de cruces</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auditoría trimestral del registro de cruces sobre una muestra de cruces, a cargo del encargado de cumplimiento del cliente (propuesta del proponente, RF-165).</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los hitos del plan de remediación instruido por la autoridad se cumplen antes de 2029.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso, con el último hito en 2029.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cumplidos antes de 2029 (Caso, cap. 7), es decir, a más tardar en el mes 24 del proyecto.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de originación de crédito, de cartera de crédito y de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operación, a más tardar en el mes 24</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe de cumplimiento por hito emitido por el proponente, que respalda el acta de la autoridad.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La cartera de 620.000 clientes con saldo migra sin pérdida, sin interrupción y sin divergencia de saldos.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plataforma de 2011 con fin de soporte en 2029.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cero diferencias sin explicar (restricción 8 del Caso).</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de cartera de crédito</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16 (primera parte) y mes 21 (segunda parte)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conciliación diaria de saldos por tramo, con registro de las diferencias y su explicación (restricción 8 del Caso).</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El evento anual se enfrenta con una estrategia de degradación definida y con capacidad de suspender la publicación de una categoría.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se improvisó durante el evento.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Orden de degradación declarado y probado (propuesta del proponente) y 104.000 pedidos en tres días (RNF-22).</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Base tecnológica y servicios de existencias y de pedidos</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16 para el orden de degradación y mes 21 para la prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En el mes 16, ensayo del orden de degradación y de la suspensión de publicación de una categoría. En el mes 21, prueba de carga de 104.000 pedidos en tres días (RNF-22).</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doña Paula sabe en qué estado está su pedido sin llamar cinco veces y, si la unidad no existe, se le avisa antes de cobrarle.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cumplimiento de la promesa de entrega en 81 %. Cinco conversaciones y nadie supo decirle qué pasó.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aviso previo al cobro (RT-16.21) y cumplimiento de la fecha de entrega sobre 97 % (Caso, cap. 7). Reclasificado desde RNF-62.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de pedidos y de existencias</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auditoría del estado único y de los avisos previos al cobro (RF-047, RF-051 y RF-052), contrastada con los contactos entrantes por el mismo caso. La parte de la solución es el estado y el aviso. La parte del cliente es el cumplimiento físico de la entrega.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compartida entre el proponente y el cliente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doña Marisol puede demostrar qué parte de la diferencia de su tienda es pérdida física y qué parte es error de registro.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todo se anota como merma y a ella se la mide por eso.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 % de las diferencias de su tienda con causa atribuida (propuesta del proponente).</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio de existencias</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 21</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revisión del informe mensual de merma con una jefatura de tienda.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Don Jonathan abre una tarjeta más rápido que hoy y el cliente recibe la información completa, sin que una cosa dependa de la otra.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tres minutos, y la información se entrega como se puede.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 segundos o menos en la evaluación y la información obligatoria antes de aceptar.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicios de originación de crédito y de evidencia financiera</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes 16</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medición comparada del tiempo de apertura y auditoría de la constancia de entrega.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proponente, con firma de la Contraparte Técnica</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>